<commit_message>
Update and Final project
</commit_message>
<xml_diff>
--- a/backend/records/AttendanceRecords.xlsx
+++ b/backend/records/AttendanceRecords.xlsx
@@ -31,28 +31,28 @@
     <t>het</t>
   </si>
   <si>
+    <t>2023031035100</t>
+  </si>
+  <si>
+    <t>Present</t>
+  </si>
+  <si>
+    <t>7/2/2026, 5:05:42 PM</t>
+  </si>
+  <si>
     <t>101</t>
   </si>
   <si>
-    <t>Present</t>
-  </si>
-  <si>
-    <t>7/8/2025, 10:49:35 am</t>
-  </si>
-  <si>
-    <t>345</t>
-  </si>
-  <si>
-    <t>7/8/2025, 7:26:21 pm</t>
-  </si>
-  <si>
-    <t>rr</t>
-  </si>
-  <si>
-    <t>12334</t>
-  </si>
-  <si>
-    <t>7/8/2025, 7:45:17 pm</t>
+    <t>7/2/2026, 5:07:31 PM</t>
+  </si>
+  <si>
+    <t>darshan</t>
+  </si>
+  <si>
+    <t>202303103510002</t>
+  </si>
+  <si>
+    <t>7/2/2026, 5:07:54 PM</t>
   </si>
 </sst>
 </file>

</xml_diff>